<commit_message>
incremental backup. defining the study selection panel in the server is basically working now.
</commit_message>
<xml_diff>
--- a/df-shorter.xlsx
+++ b/df-shorter.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dallbrit\OneDrive - DePaul University\Documents\R Projects\shiny-meta-development\newShinyMeta\Code\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://depauledu-my.sharepoint.com/personal/dallbrit_depaul_edu/Documents/Documents/R Projects/shiny-meta-development/newShinyMeta/Code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{23A7649D-4511-455F-92A1-0422556ACA87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{23A7649D-4511-455F-92A1-0422556ACA87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2676C5FA-BAD5-4AEA-AEC0-A979EAB18377}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="80">
   <si>
     <t>yi</t>
   </si>
@@ -257,6 +257,9 @@
   </si>
   <si>
     <t>lyrical</t>
+  </si>
+  <si>
+    <t>Anderson &amp; fakeName for debugging (2010)</t>
   </si>
 </sst>
 </file>
@@ -1786,7 +1789,7 @@
         <v>1</v>
       </c>
       <c r="G12" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="H12" t="s">
         <v>76</v>

</xml_diff>